<commit_message>
fix(cascada): blindaje inmediato de cuarentena en vivo y reseteo estricto a linea media
</commit_message>
<xml_diff>
--- a/ReportesTrades/Tabla_Maestra_Consolidada_Tabla dinamica.xlsx
+++ b/ReportesTrades/Tabla_Maestra_Consolidada_Tabla dinamica.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Documents\NinjaTrader 8\bin\Custom\ReportesTrades\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4F32D94-EAFE-4D1A-8601-B9F99E17064D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4E6CAF-FEE5-4150-AFA9-28E5C350AD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{8E15BEA4-5177-40D5-87FF-3C71603A24EE}"/>
+    <workbookView xWindow="29970" yWindow="1200" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8E15BEA4-5177-40D5-87FF-3C71603A24EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Base_Trades" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -341,14 +341,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -486,6 +485,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
       <x14:pivotCacheDefinition/>
+    </ext>
+    <ext xmlns:xlpdsc="http://schemas.microsoft.com/office/spreadsheetml/2026/pivotDataSourceClean" uri="{F4336242-56EE-4DD3-A5F7-E900642BF6E9}">
+      <xlpdsc:dataSourceClean>1</xlpdsc:dataSourceClean>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -1141,7 +1143,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F8080E09-DC14-4D51-B8B4-A148AA69EA0B}" name="TablaDinámica2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F8080E09-DC14-4D51-B8B4-A148AA69EA0B}" name="TablaDinámica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="I1:S5" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisCol" numFmtId="14" showAll="0">
@@ -1234,7 +1236,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C689540E-A3B9-43B7-A05A-C9EEF4CD6557}" name="Tabla2" displayName="Tabla2" ref="A1:Y235" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C689540E-A3B9-43B7-A05A-C9EEF4CD6557}" name="Tabla2" displayName="Tabla2" ref="A1:Y235" totalsRowShown="0" headerRowDxfId="14">
   <autoFilter ref="A1:Y235" xr:uid="{C689540E-A3B9-43B7-A05A-C9EEF4CD6557}">
     <filterColumn colId="0">
       <filters>
@@ -1247,6 +1249,11 @@
         <filter val="NTSniperSurfer10202026.xlsx"/>
         <filter val="NTSniperSurfer10212026.xlsx"/>
         <filter val="NTSniperSurfer10222026.xlsx"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <dateGroupItem year="2026" month="10" day="19" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -1282,7 +1289,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F3A4D07E-BED8-41CC-B08C-FA56A74D83B5}" name="Tabla1" displayName="Tabla1" ref="A1:E7271" totalsRowShown="0" headerRowDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F3A4D07E-BED8-41CC-B08C-FA56A74D83B5}" name="Tabla1" displayName="Tabla1" ref="A1:E7271" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:E7271" xr:uid="{F3A4D07E-BED8-41CC-B08C-FA56A74D83B5}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{58DD40C9-7EB7-4682-993E-972FFA85F277}" name="Fecha"/>
@@ -1618,17 +1625,16 @@
     <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5703125" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="12" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="6.28515625" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="18.85546875" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="25.140625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16.85546875" customWidth="1"/>
     <col min="17" max="17" width="14.5703125" customWidth="1"/>
@@ -1636,8 +1642,9 @@
     <col min="19" max="19" width="15.42578125" hidden="1" customWidth="1"/>
     <col min="20" max="20" width="8.5703125" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="10.42578125" hidden="1" customWidth="1"/>
-    <col min="22" max="24" width="8.28515625" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="7" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="8.28515625" hidden="1" customWidth="1"/>
+    <col min="23" max="24" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="7.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
@@ -12801,7 +12808,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="150" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>55</v>
       </c>
@@ -12877,9 +12884,9 @@
       <c r="Y150">
         <v>32</v>
       </c>
-      <c r="Z150" s="8"/>
-    </row>
-    <row r="151" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z150" s="7"/>
+    </row>
+    <row r="151" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>55</v>
       </c>
@@ -12955,9 +12962,9 @@
       <c r="Y151">
         <v>40</v>
       </c>
-      <c r="Z151" s="8"/>
-    </row>
-    <row r="152" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z151" s="7"/>
+    </row>
+    <row r="152" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>55</v>
       </c>
@@ -13033,9 +13040,9 @@
       <c r="Y152">
         <v>40</v>
       </c>
-      <c r="Z152" s="8"/>
-    </row>
-    <row r="153" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z152" s="7"/>
+    </row>
+    <row r="153" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>55</v>
       </c>
@@ -13111,9 +13118,9 @@
       <c r="Y153">
         <v>36</v>
       </c>
-      <c r="Z153" s="8"/>
-    </row>
-    <row r="154" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z153" s="7"/>
+    </row>
+    <row r="154" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>55</v>
       </c>
@@ -13189,9 +13196,9 @@
       <c r="Y154">
         <v>29</v>
       </c>
-      <c r="Z154" s="8"/>
-    </row>
-    <row r="155" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z154" s="7"/>
+    </row>
+    <row r="155" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>61</v>
       </c>
@@ -13267,9 +13274,9 @@
       <c r="Y155">
         <v>44</v>
       </c>
-      <c r="Z155" s="9"/>
-    </row>
-    <row r="156" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z155" s="8"/>
+    </row>
+    <row r="156" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>61</v>
       </c>
@@ -13345,9 +13352,9 @@
       <c r="Y156">
         <v>6</v>
       </c>
-      <c r="Z156" s="9"/>
-    </row>
-    <row r="157" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z156" s="8"/>
+    </row>
+    <row r="157" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>61</v>
       </c>
@@ -13423,9 +13430,9 @@
       <c r="Y157">
         <v>47</v>
       </c>
-      <c r="Z157" s="9"/>
-    </row>
-    <row r="158" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z157" s="8"/>
+    </row>
+    <row r="158" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>61</v>
       </c>
@@ -13501,9 +13508,9 @@
       <c r="Y158">
         <v>24</v>
       </c>
-      <c r="Z158" s="9"/>
-    </row>
-    <row r="159" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z158" s="8"/>
+    </row>
+    <row r="159" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>61</v>
       </c>
@@ -13579,9 +13586,9 @@
       <c r="Y159">
         <v>22</v>
       </c>
-      <c r="Z159" s="9"/>
-    </row>
-    <row r="160" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z159" s="8"/>
+    </row>
+    <row r="160" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>61</v>
       </c>
@@ -13657,9 +13664,9 @@
       <c r="Y160">
         <v>57</v>
       </c>
-      <c r="Z160" s="9"/>
-    </row>
-    <row r="161" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z160" s="8"/>
+    </row>
+    <row r="161" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>61</v>
       </c>
@@ -13735,9 +13742,9 @@
       <c r="Y161">
         <v>21</v>
       </c>
-      <c r="Z161" s="9"/>
-    </row>
-    <row r="162" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z161" s="8"/>
+    </row>
+    <row r="162" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>61</v>
       </c>
@@ -13813,9 +13820,9 @@
       <c r="Y162">
         <v>32</v>
       </c>
-      <c r="Z162" s="9"/>
-    </row>
-    <row r="163" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z162" s="8"/>
+    </row>
+    <row r="163" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>61</v>
       </c>
@@ -13891,9 +13898,9 @@
       <c r="Y163">
         <v>13</v>
       </c>
-      <c r="Z163" s="9"/>
-    </row>
-    <row r="164" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z163" s="8"/>
+    </row>
+    <row r="164" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>61</v>
       </c>
@@ -13969,9 +13976,9 @@
       <c r="Y164">
         <v>27</v>
       </c>
-      <c r="Z164" s="9"/>
-    </row>
-    <row r="165" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z164" s="8"/>
+    </row>
+    <row r="165" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>63</v>
       </c>
@@ -14047,9 +14054,9 @@
       <c r="Y165">
         <v>30</v>
       </c>
-      <c r="Z165" s="10"/>
-    </row>
-    <row r="166" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z165" s="9"/>
+    </row>
+    <row r="166" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>63</v>
       </c>
@@ -14125,9 +14132,9 @@
       <c r="Y166">
         <v>11</v>
       </c>
-      <c r="Z166" s="10"/>
-    </row>
-    <row r="167" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z166" s="9"/>
+    </row>
+    <row r="167" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>63</v>
       </c>
@@ -14203,9 +14210,9 @@
       <c r="Y167">
         <v>32</v>
       </c>
-      <c r="Z167" s="10"/>
-    </row>
-    <row r="168" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z167" s="9"/>
+    </row>
+    <row r="168" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>63</v>
       </c>
@@ -14281,9 +14288,9 @@
       <c r="Y168">
         <v>37</v>
       </c>
-      <c r="Z168" s="10"/>
-    </row>
-    <row r="169" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z168" s="9"/>
+    </row>
+    <row r="169" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>63</v>
       </c>
@@ -14359,9 +14366,9 @@
       <c r="Y169">
         <v>28</v>
       </c>
-      <c r="Z169" s="10"/>
-    </row>
-    <row r="170" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z169" s="9"/>
+    </row>
+    <row r="170" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>63</v>
       </c>
@@ -14437,9 +14444,9 @@
       <c r="Y170">
         <v>8</v>
       </c>
-      <c r="Z170" s="10"/>
-    </row>
-    <row r="171" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z170" s="9"/>
+    </row>
+    <row r="171" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>63</v>
       </c>
@@ -14515,9 +14522,9 @@
       <c r="Y171">
         <v>9</v>
       </c>
-      <c r="Z171" s="10"/>
-    </row>
-    <row r="172" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z171" s="9"/>
+    </row>
+    <row r="172" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>63</v>
       </c>
@@ -14593,9 +14600,9 @@
       <c r="Y172">
         <v>53</v>
       </c>
-      <c r="Z172" s="10"/>
-    </row>
-    <row r="173" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z172" s="9"/>
+    </row>
+    <row r="173" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>63</v>
       </c>
@@ -14671,9 +14678,9 @@
       <c r="Y173">
         <v>8</v>
       </c>
-      <c r="Z173" s="10"/>
-    </row>
-    <row r="174" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z173" s="9"/>
+    </row>
+    <row r="174" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>63</v>
       </c>
@@ -14749,9 +14756,9 @@
       <c r="Y174">
         <v>37</v>
       </c>
-      <c r="Z174" s="10"/>
-    </row>
-    <row r="175" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z174" s="9"/>
+    </row>
+    <row r="175" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>63</v>
       </c>
@@ -14827,9 +14834,9 @@
       <c r="Y175">
         <v>36</v>
       </c>
-      <c r="Z175" s="10"/>
-    </row>
-    <row r="176" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z175" s="9"/>
+    </row>
+    <row r="176" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>63</v>
       </c>
@@ -14905,9 +14912,9 @@
       <c r="Y176">
         <v>24</v>
       </c>
-      <c r="Z176" s="10"/>
-    </row>
-    <row r="177" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z176" s="9"/>
+    </row>
+    <row r="177" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>64</v>
       </c>
@@ -14983,9 +14990,9 @@
       <c r="Y177">
         <v>3</v>
       </c>
-      <c r="Z177" s="8"/>
-    </row>
-    <row r="178" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z177" s="7"/>
+    </row>
+    <row r="178" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>64</v>
       </c>
@@ -15061,9 +15068,9 @@
       <c r="Y178">
         <v>23</v>
       </c>
-      <c r="Z178" s="8"/>
-    </row>
-    <row r="179" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z178" s="7"/>
+    </row>
+    <row r="179" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>64</v>
       </c>
@@ -15139,9 +15146,9 @@
       <c r="Y179">
         <v>4</v>
       </c>
-      <c r="Z179" s="8"/>
-    </row>
-    <row r="180" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z179" s="7"/>
+    </row>
+    <row r="180" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>64</v>
       </c>
@@ -15217,9 +15224,9 @@
       <c r="Y180">
         <v>17</v>
       </c>
-      <c r="Z180" s="8"/>
-    </row>
-    <row r="181" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z180" s="7"/>
+    </row>
+    <row r="181" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>64</v>
       </c>
@@ -15295,9 +15302,9 @@
       <c r="Y181">
         <v>30</v>
       </c>
-      <c r="Z181" s="8"/>
-    </row>
-    <row r="182" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z181" s="7"/>
+    </row>
+    <row r="182" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>64</v>
       </c>
@@ -15373,9 +15380,9 @@
       <c r="Y182">
         <v>11</v>
       </c>
-      <c r="Z182" s="8"/>
-    </row>
-    <row r="183" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z182" s="7"/>
+    </row>
+    <row r="183" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>64</v>
       </c>
@@ -15451,9 +15458,9 @@
       <c r="Y183">
         <v>31</v>
       </c>
-      <c r="Z183" s="8"/>
-    </row>
-    <row r="184" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z183" s="7"/>
+    </row>
+    <row r="184" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>65</v>
       </c>
@@ -15529,9 +15536,9 @@
       <c r="Y184">
         <v>22</v>
       </c>
-      <c r="Z184" s="9"/>
-    </row>
-    <row r="185" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z184" s="8"/>
+    </row>
+    <row r="185" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>65</v>
       </c>
@@ -15607,9 +15614,9 @@
       <c r="Y185">
         <v>19</v>
       </c>
-      <c r="Z185" s="9"/>
-    </row>
-    <row r="186" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z185" s="8"/>
+    </row>
+    <row r="186" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>65</v>
       </c>
@@ -15685,9 +15692,9 @@
       <c r="Y186">
         <v>10</v>
       </c>
-      <c r="Z186" s="9"/>
-    </row>
-    <row r="187" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z186" s="8"/>
+    </row>
+    <row r="187" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>65</v>
       </c>
@@ -15763,9 +15770,9 @@
       <c r="Y187">
         <v>40</v>
       </c>
-      <c r="Z187" s="9"/>
-    </row>
-    <row r="188" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z187" s="8"/>
+    </row>
+    <row r="188" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>65</v>
       </c>
@@ -15841,9 +15848,9 @@
       <c r="Y188">
         <v>36</v>
       </c>
-      <c r="Z188" s="9"/>
-    </row>
-    <row r="189" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z188" s="8"/>
+    </row>
+    <row r="189" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>65</v>
       </c>
@@ -15919,9 +15926,9 @@
       <c r="Y189">
         <v>3</v>
       </c>
-      <c r="Z189" s="9"/>
-    </row>
-    <row r="190" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z189" s="8"/>
+    </row>
+    <row r="190" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>65</v>
       </c>
@@ -15997,9 +16004,9 @@
       <c r="Y190">
         <v>23</v>
       </c>
-      <c r="Z190" s="9"/>
-    </row>
-    <row r="191" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z190" s="8"/>
+    </row>
+    <row r="191" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>65</v>
       </c>
@@ -16075,9 +16082,9 @@
       <c r="Y191">
         <v>4</v>
       </c>
-      <c r="Z191" s="9"/>
-    </row>
-    <row r="192" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z191" s="8"/>
+    </row>
+    <row r="192" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>65</v>
       </c>
@@ -16153,9 +16160,9 @@
       <c r="Y192">
         <v>6</v>
       </c>
-      <c r="Z192" s="9"/>
-    </row>
-    <row r="193" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z192" s="8"/>
+    </row>
+    <row r="193" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>65</v>
       </c>
@@ -16231,9 +16238,9 @@
       <c r="Y193">
         <v>37</v>
       </c>
-      <c r="Z193" s="9"/>
-    </row>
-    <row r="194" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z193" s="8"/>
+    </row>
+    <row r="194" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>65</v>
       </c>
@@ -16309,9 +16316,9 @@
       <c r="Y194">
         <v>5</v>
       </c>
-      <c r="Z194" s="9"/>
-    </row>
-    <row r="195" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z194" s="8"/>
+    </row>
+    <row r="195" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>65</v>
       </c>
@@ -16387,9 +16394,9 @@
       <c r="Y195">
         <v>24</v>
       </c>
-      <c r="Z195" s="9"/>
-    </row>
-    <row r="196" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z195" s="8"/>
+    </row>
+    <row r="196" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>65</v>
       </c>
@@ -16465,9 +16472,9 @@
       <c r="Y196">
         <v>3</v>
       </c>
-      <c r="Z196" s="9"/>
-    </row>
-    <row r="197" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z196" s="8"/>
+    </row>
+    <row r="197" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>65</v>
       </c>
@@ -16543,9 +16550,9 @@
       <c r="Y197">
         <v>16</v>
       </c>
-      <c r="Z197" s="9"/>
-    </row>
-    <row r="198" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z197" s="8"/>
+    </row>
+    <row r="198" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>65</v>
       </c>
@@ -16621,7 +16628,7 @@
       <c r="Y198">
         <v>36</v>
       </c>
-      <c r="Z198" s="9"/>
+      <c r="Z198" s="8"/>
     </row>
     <row r="199" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
@@ -16699,7 +16706,7 @@
       <c r="Y199">
         <v>17</v>
       </c>
-      <c r="Z199" s="10"/>
+      <c r="Z199" s="9"/>
     </row>
     <row r="200" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
@@ -16777,7 +16784,7 @@
       <c r="Y200">
         <v>26</v>
       </c>
-      <c r="Z200" s="10"/>
+      <c r="Z200" s="9"/>
     </row>
     <row r="201" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
@@ -16855,7 +16862,7 @@
       <c r="Y201">
         <v>10</v>
       </c>
-      <c r="Z201" s="10"/>
+      <c r="Z201" s="9"/>
     </row>
     <row r="202" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
@@ -16933,7 +16940,7 @@
       <c r="Y202">
         <v>32</v>
       </c>
-      <c r="Z202" s="10"/>
+      <c r="Z202" s="9"/>
     </row>
     <row r="203" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
@@ -17011,7 +17018,7 @@
       <c r="Y203">
         <v>9</v>
       </c>
-      <c r="Z203" s="10"/>
+      <c r="Z203" s="9"/>
     </row>
     <row r="204" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
@@ -17089,7 +17096,7 @@
       <c r="Y204">
         <v>21</v>
       </c>
-      <c r="Z204" s="10"/>
+      <c r="Z204" s="9"/>
     </row>
     <row r="205" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
@@ -17167,9 +17174,9 @@
       <c r="Y205">
         <v>8</v>
       </c>
-      <c r="Z205" s="10"/>
-    </row>
-    <row r="206" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z205" s="9"/>
+    </row>
+    <row r="206" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>67</v>
       </c>
@@ -17245,9 +17252,9 @@
       <c r="Y206">
         <v>17</v>
       </c>
-      <c r="Z206" s="8"/>
-    </row>
-    <row r="207" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z206" s="7"/>
+    </row>
+    <row r="207" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>67</v>
       </c>
@@ -17323,9 +17330,9 @@
       <c r="Y207">
         <v>33</v>
       </c>
-      <c r="Z207" s="8"/>
-    </row>
-    <row r="208" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z207" s="7"/>
+    </row>
+    <row r="208" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>67</v>
       </c>
@@ -17401,9 +17408,9 @@
       <c r="Y208">
         <v>37</v>
       </c>
-      <c r="Z208" s="8"/>
-    </row>
-    <row r="209" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z208" s="7"/>
+    </row>
+    <row r="209" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>67</v>
       </c>
@@ -17479,9 +17486,9 @@
       <c r="Y209">
         <v>4</v>
       </c>
-      <c r="Z209" s="8"/>
-    </row>
-    <row r="210" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z209" s="7"/>
+    </row>
+    <row r="210" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>67</v>
       </c>
@@ -17557,9 +17564,9 @@
       <c r="Y210">
         <v>38</v>
       </c>
-      <c r="Z210" s="8"/>
-    </row>
-    <row r="211" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z210" s="7"/>
+    </row>
+    <row r="211" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>67</v>
       </c>
@@ -17635,9 +17642,9 @@
       <c r="Y211">
         <v>53</v>
       </c>
-      <c r="Z211" s="8"/>
-    </row>
-    <row r="212" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z211" s="7"/>
+    </row>
+    <row r="212" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>67</v>
       </c>
@@ -17713,9 +17720,9 @@
       <c r="Y212">
         <v>29</v>
       </c>
-      <c r="Z212" s="8"/>
-    </row>
-    <row r="213" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z212" s="7"/>
+    </row>
+    <row r="213" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>67</v>
       </c>
@@ -17791,9 +17798,9 @@
       <c r="Y213">
         <v>18</v>
       </c>
-      <c r="Z213" s="8"/>
-    </row>
-    <row r="214" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z213" s="7"/>
+    </row>
+    <row r="214" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>68</v>
       </c>
@@ -17869,9 +17876,9 @@
       <c r="Y214">
         <v>36</v>
       </c>
-      <c r="Z214" s="9"/>
-    </row>
-    <row r="215" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z214" s="8"/>
+    </row>
+    <row r="215" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>68</v>
       </c>
@@ -17947,9 +17954,9 @@
       <c r="Y215">
         <v>20</v>
       </c>
-      <c r="Z215" s="9"/>
-    </row>
-    <row r="216" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z215" s="8"/>
+    </row>
+    <row r="216" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>68</v>
       </c>
@@ -18025,9 +18032,9 @@
       <c r="Y216">
         <v>22</v>
       </c>
-      <c r="Z216" s="9"/>
-    </row>
-    <row r="217" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z216" s="8"/>
+    </row>
+    <row r="217" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>68</v>
       </c>
@@ -18103,9 +18110,9 @@
       <c r="Y217">
         <v>22</v>
       </c>
-      <c r="Z217" s="9"/>
-    </row>
-    <row r="218" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z217" s="8"/>
+    </row>
+    <row r="218" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>68</v>
       </c>
@@ -18181,9 +18188,9 @@
       <c r="Y218">
         <v>23</v>
       </c>
-      <c r="Z218" s="9"/>
-    </row>
-    <row r="219" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z218" s="8"/>
+    </row>
+    <row r="219" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>68</v>
       </c>
@@ -18259,9 +18266,9 @@
       <c r="Y219">
         <v>10</v>
       </c>
-      <c r="Z219" s="9"/>
-    </row>
-    <row r="220" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z219" s="8"/>
+    </row>
+    <row r="220" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>68</v>
       </c>
@@ -18337,9 +18344,9 @@
       <c r="Y220">
         <v>25</v>
       </c>
-      <c r="Z220" s="9"/>
-    </row>
-    <row r="221" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z220" s="8"/>
+    </row>
+    <row r="221" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>68</v>
       </c>
@@ -18415,9 +18422,9 @@
       <c r="Y221">
         <v>7</v>
       </c>
-      <c r="Z221" s="9"/>
-    </row>
-    <row r="222" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z221" s="8"/>
+    </row>
+    <row r="222" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>69</v>
       </c>
@@ -18493,9 +18500,9 @@
       <c r="Y222">
         <v>43</v>
       </c>
-      <c r="Z222" s="10"/>
-    </row>
-    <row r="223" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z222" s="9"/>
+    </row>
+    <row r="223" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>69</v>
       </c>
@@ -18571,9 +18578,9 @@
       <c r="Y223">
         <v>7</v>
       </c>
-      <c r="Z223" s="10"/>
-    </row>
-    <row r="224" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z223" s="9"/>
+    </row>
+    <row r="224" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>69</v>
       </c>
@@ -18649,9 +18656,9 @@
       <c r="Y224">
         <v>36</v>
       </c>
-      <c r="Z224" s="10"/>
-    </row>
-    <row r="225" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z224" s="9"/>
+    </row>
+    <row r="225" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>69</v>
       </c>
@@ -18727,9 +18734,9 @@
       <c r="Y225">
         <v>23</v>
       </c>
-      <c r="Z225" s="10"/>
-    </row>
-    <row r="226" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z225" s="9"/>
+    </row>
+    <row r="226" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>69</v>
       </c>
@@ -18805,9 +18812,9 @@
       <c r="Y226">
         <v>6</v>
       </c>
-      <c r="Z226" s="10"/>
-    </row>
-    <row r="227" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z226" s="9"/>
+    </row>
+    <row r="227" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>69</v>
       </c>
@@ -18883,9 +18890,9 @@
       <c r="Y227">
         <v>21</v>
       </c>
-      <c r="Z227" s="10"/>
-    </row>
-    <row r="228" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z227" s="9"/>
+    </row>
+    <row r="228" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>69</v>
       </c>
@@ -18961,9 +18968,9 @@
       <c r="Y228">
         <v>18</v>
       </c>
-      <c r="Z228" s="10"/>
-    </row>
-    <row r="229" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z228" s="9"/>
+    </row>
+    <row r="229" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>69</v>
       </c>
@@ -19039,9 +19046,9 @@
       <c r="Y229">
         <v>25</v>
       </c>
-      <c r="Z229" s="10"/>
-    </row>
-    <row r="230" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z229" s="9"/>
+    </row>
+    <row r="230" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>69</v>
       </c>
@@ -19117,9 +19124,9 @@
       <c r="Y230">
         <v>40</v>
       </c>
-      <c r="Z230" s="10"/>
-    </row>
-    <row r="231" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z230" s="9"/>
+    </row>
+    <row r="231" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>69</v>
       </c>
@@ -19195,9 +19202,9 @@
       <c r="Y231">
         <v>22</v>
       </c>
-      <c r="Z231" s="10"/>
-    </row>
-    <row r="232" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z231" s="9"/>
+    </row>
+    <row r="232" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>69</v>
       </c>
@@ -19273,9 +19280,9 @@
       <c r="Y232">
         <v>27</v>
       </c>
-      <c r="Z232" s="10"/>
-    </row>
-    <row r="233" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z232" s="9"/>
+    </row>
+    <row r="233" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>69</v>
       </c>
@@ -19351,9 +19358,9 @@
       <c r="Y233">
         <v>33</v>
       </c>
-      <c r="Z233" s="10"/>
-    </row>
-    <row r="234" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z233" s="9"/>
+    </row>
+    <row r="234" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>69</v>
       </c>
@@ -19429,9 +19436,9 @@
       <c r="Y234">
         <v>22</v>
       </c>
-      <c r="Z234" s="10"/>
-    </row>
-    <row r="235" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Z234" s="9"/>
+    </row>
+    <row r="235" spans="1:26" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>69</v>
       </c>
@@ -19507,7 +19514,7 @@
       <c r="Y235">
         <v>21</v>
       </c>
-      <c r="Z235" s="10"/>
+      <c r="Z235" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19632,37 +19639,37 @@
       <c r="E3">
         <v>16.28</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3">
         <v>123.83999999999999</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3">
         <v>-636.04</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3">
         <v>145.93999999999994</v>
       </c>
-      <c r="M3" s="6">
+      <c r="M3">
         <v>280.23999999999995</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3">
         <v>674.72</v>
       </c>
-      <c r="O3" s="6">
+      <c r="O3">
         <v>1155.2400000000002</v>
       </c>
-      <c r="P3" s="6">
+      <c r="P3">
         <v>297.09999999999985</v>
       </c>
-      <c r="Q3" s="6">
+      <c r="Q3">
         <v>377.03999999999985</v>
       </c>
-      <c r="R3" s="6">
+      <c r="R3">
         <v>-375.8599999999999</v>
       </c>
-      <c r="S3" s="6">
+      <c r="S3">
         <v>2042.22</v>
       </c>
     </row>
@@ -19682,37 +19689,37 @@
       <c r="E4">
         <v>145.63999999999999</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4">
         <v>-21.799999999999997</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4">
         <v>-943.6</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4">
         <v>-964.82</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4">
         <v>806.9799999999999</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4">
         <v>9.5999999999999943</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4">
         <v>481.9799999999999</v>
       </c>
-      <c r="P4" s="6">
+      <c r="P4">
         <v>677.61999999999989</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="Q4">
         <v>590.11999999999989</v>
       </c>
-      <c r="R4" s="6">
+      <c r="R4">
         <v>963.96</v>
       </c>
-      <c r="S4" s="6">
+      <c r="S4">
         <v>1600.0399999999995</v>
       </c>
     </row>
@@ -19732,37 +19739,37 @@
       <c r="E5">
         <v>-16.86</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5">
         <v>102.03999999999999</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5">
         <v>-1579.6399999999999</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5">
         <v>-818.88000000000011</v>
       </c>
-      <c r="M5" s="6">
+      <c r="M5">
         <v>1087.2199999999998</v>
       </c>
-      <c r="N5" s="6">
+      <c r="N5">
         <v>684.32</v>
       </c>
-      <c r="O5" s="6">
+      <c r="O5">
         <v>1637.2200000000003</v>
       </c>
-      <c r="P5" s="6">
+      <c r="P5">
         <v>974.7199999999998</v>
       </c>
-      <c r="Q5" s="6">
+      <c r="Q5">
         <v>967.15999999999974</v>
       </c>
-      <c r="R5" s="6">
+      <c r="R5">
         <v>588.10000000000014</v>
       </c>
-      <c r="S5" s="6">
+      <c r="S5">
         <v>3642.2599999999993</v>
       </c>
     </row>

</xml_diff>